<commit_message>
feat: Add generar ticket errores and new modules
</commit_message>
<xml_diff>
--- a/GENERAL_BOTS.xlsx
+++ b/GENERAL_BOTS.xlsx
@@ -402,15 +402,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G8"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -561,7 +552,7 @@
         <v>800229362</v>
       </c>
       <c r="D7">
-        <v>11025232024</v>
+        <v>11027492024</v>
       </c>
       <c r="E7" t="str">
         <v>2024</v>
@@ -606,13 +597,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E60"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>